<commit_message>
Run OpenAI extraction on all confirmations and refine receipt-only/EUR fields in Python.
The API path now extracts 31 native-text PDFs and 4 Continental scans via vision. Deterministic post-processing classifies Liberty no-schedule acks and fills Ostmark prices that are printed on the PDF without inventing omitted PO lines.

Co-authored-by: anthonyleedu <anthonyleedu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/follow_up_drafts.xlsx
+++ b/output/follow_up_drafts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
   <si>
     <t>Vendor</t>
   </si>
@@ -84,6 +84,9 @@
 Thank you.
 Lisa Morgan
 Purchasing, Beacon Fasteners</t>
+  </si>
+  <si>
+    <t>APEX BAR &amp; TUBE CO.</t>
   </si>
   <si>
     <t>PO-4500060619</t>
@@ -646,19 +649,19 @@
     </row>
     <row r="6" spans="1:5" ht="90" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="90" customHeight="1">
@@ -669,81 +672,81 @@
         <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="90" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="90" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="90" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="90" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Polish monthly PARTIAL labels, combine PO-level follow-ups, and clarify revision codes.
Mark 2025-09 and 2026-05 as partial months, emit one QuickShip invoice follow-up covering both lines, and rename DOCUMENT_SUPERSEDED on active rows to PRIOR_DOCUMENT_SUPERSEDED. Core OTD, spend, and exception counts are unchanged.

Co-authored-by: anthonyleedu <anthonyleedu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/follow_up_drafts.xlsx
+++ b/output/follow_up_drafts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
   <si>
     <t>Vendor</t>
   </si>
@@ -45,7 +45,7 @@
   <si>
     <t>Hello,
 We received your document for PO-4500050001.
-Beacon PO PO-4500050001 line 2 (BAR-A286-250, qty 1,500 if ordered, required 2026-06-10) does not appear on the acknowledgment. Please confirm this line.
+Beacon PO PO-4500050001 line 2 BAR-A286-250 (BAR-A286-250, qty 1,500 if ordered, required 2026-06-10) does not appear on the acknowledgment. Please confirm this line.
 Thank you.
 Lisa Morgan
 Purchasing, Beacon Fasteners</t>
@@ -75,12 +75,13 @@
     <t>PO-4500050032</t>
   </si>
   <si>
-    <t>PO-4500050032 confirmation discrepancy</t>
+    <t>PO-4500050032 formal acknowledgment requested</t>
   </si>
   <si>
     <t>Hello,
 We received your document for PO-4500050032.
-We have shipment/invoice evidence for PO-4500050032 but no formal order acknowledgment. Please send a confirmation of quantity, price, and promise date.
+Beacon has an invoice or shipping document for PO-4500050032, but no formal order acknowledgment.
+Please confirm quantity, price, and commitment date for line 1 MISC-WAS-A25 and line 2 MISC-SPR-001.
 Thank you.
 Lisa Morgan
 Purchasing, Beacon Fasteners</t>
@@ -185,7 +186,7 @@
   <si>
     <t>Hello,
 We received your document for PO-4500050019.
-Please provide a committed quantity and promise date for PO-4500050019 line 1 (PLAT-PASV).
+Please provide a committed quantity and promise date for PO-4500050019 line 1 PLAT-PASV.
 Thank you.
 Lisa Morgan
 Purchasing, Beacon Fasteners</t>
@@ -553,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="28.7109375" customWidth="1"/>
@@ -632,87 +633,87 @@
     </row>
     <row r="5" spans="1:5" ht="90" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="90" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="90" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="90" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="90" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="90" customHeight="1">
@@ -723,29 +724,12 @@
         <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="90" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" s="2" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>